<commit_message>
refactor get all resume, add campo idBoard e create sem mostrar erro
</commit_message>
<xml_diff>
--- a/base/beercapboard.xlsx
+++ b/base/beercapboard.xlsx
@@ -4,21 +4,28 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8130"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8130" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="beercapboard" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="beer" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="beercapboard" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
   <si>
+    <t>id_board</t>
+  </si>
+  <si>
+    <t>posicao</t>
+  </si>
+  <si>
     <t>data_consumo</t>
   </si>
   <si>
@@ -34,7 +41,7 @@
     <t>comentarios</t>
   </si>
   <si>
-    <t>beerCapColor</t>
+    <t>beer_cap_color</t>
   </si>
   <si>
     <t>Interestellar</t>
@@ -61,9 +68,6 @@
     <t>orange</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>02/02/2020</t>
   </si>
   <si>
@@ -79,16 +83,19 @@
     <t>#fb2323</t>
   </si>
   <si>
+    <t>id_user</t>
+  </si>
+  <si>
+    <t>Mario</t>
+  </si>
+  <si>
+    <t>IPA maracujá</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>01/01/2020</t>
-  </si>
-  <si>
-    <t>boa, leve</t>
-  </si>
-  <si>
-    <t>#678ad0</t>
+    <t>#d829db</t>
   </si>
 </sst>
 </file>
@@ -472,17 +479,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="6" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="1" max="3" width="10" customWidth="1"/>
+    <col min="4" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -504,19 +511,25 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>3</v>
       </c>
-      <c r="B2" s="1">
+      <c r="D2" s="1">
         <v>45253</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
@@ -527,36 +540,51 @@
       <c r="G2" t="s">
         <v>11</v>
       </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
         <v>5</v>
       </c>
-      <c r="B3" s="1">
+      <c r="D3" s="1">
         <v>45983</v>
       </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
       <c r="E3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
       </c>
       <c r="D4" t="s">
         <v>17</v>
@@ -565,40 +593,78 @@
         <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="I4" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="2" x14ac:dyDescent="0" defaultColWidth="8.72727272727273" customHeight="1"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ajuste create back e front; atualizacao automatica board
</commit_message>
<xml_diff>
--- a/base/beercapboard.xlsx
+++ b/base/beercapboard.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8130" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8130"/>
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="beer" state="visible" r:id="rId4"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
   <si>
     <t>id</t>
   </si>
@@ -83,19 +83,73 @@
     <t>#fb2323</t>
   </si>
   <si>
+    <t>2025-11-25</t>
+  </si>
+  <si>
+    <t>Paulaner Weissbier</t>
+  </si>
+  <si>
+    <t>Paulaner Munichen</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>saborosa</t>
+  </si>
+  <si>
+    <t>#e8d86d</t>
+  </si>
+  <si>
+    <t>2025-11-19</t>
+  </si>
+  <si>
+    <t>Iron Maiden</t>
+  </si>
+  <si>
+    <t>Trooper</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>pesada</t>
+  </si>
+  <si>
+    <t>#000000</t>
+  </si>
+  <si>
+    <t>Praya Wit</t>
+  </si>
+  <si>
+    <t>Praya</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>#51c6c8</t>
+  </si>
+  <si>
+    <t>2025-11-05</t>
+  </si>
+  <si>
+    <t>teste</t>
+  </si>
+  <si>
+    <t>st3s</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>#00ff4c</t>
+  </si>
+  <si>
     <t>id_user</t>
   </si>
   <si>
     <t>Mario</t>
-  </si>
-  <si>
-    <t>IPA maracujá</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>#d829db</t>
   </si>
 </sst>
 </file>
@@ -479,8 +533,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="4" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="9" customHeight="1"/>
   <cols>
     <col min="1" max="3" width="10" customWidth="1"/>
     <col min="4" max="6" width="25" customWidth="1"/>
@@ -605,6 +659,122 @@
         <v>21</v>
       </c>
     </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -613,7 +783,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="2" x14ac:dyDescent="0" defaultColWidth="8.72727272727273" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -621,7 +791,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
         <v>4</v>
@@ -635,33 +805,7 @@
         <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>7</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>